<commit_message>
Set payslip template to 3,800 EUR gross monthly salary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjpH9z1P7SfaWGA8PX7UuE
</commit_message>
<xml_diff>
--- a/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
+++ b/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
@@ -250,7 +250,7 @@
   <commentList>
     <comment ref="B22" authorId="0" shapeId="0">
       <text>
-        <t>Fila de ejemplo (30 días x 40 €). Sustitúyela por los datos reales.</t>
+        <t>Salario bruto mensual de 3.800 €. Si se reparte en varios conceptos (complementos, prorrata de pagas), ajusta estas filas para que sumen lo pactado en el contrato.</t>
       </text>
     </comment>
     <comment ref="B28" authorId="0" shapeId="0">
@@ -285,7 +285,7 @@
     </comment>
     <comment ref="D43" authorId="0" shapeId="0">
       <text>
-        <t>Porcentaje de ejemplo. Calcular con el simulador de retenciones de la AEAT según la situación del trabajador.</t>
+        <t>18 % orientativo. Calcular con el simulador de retenciones de la AEAT según la situación del trabajador.</t>
       </text>
     </comment>
   </commentList>
@@ -888,14 +888,14 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Salario base</t>
+          <t>Salario base mensual</t>
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D22" s="14" t="n">
-        <v>40</v>
+        <v>3800</v>
       </c>
       <c r="E22" s="15">
         <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),C22*D22,0)</f>
@@ -1327,7 +1327,7 @@
         <v/>
       </c>
       <c r="D43" s="20" t="n">
-        <v>0.02</v>
+        <v>0.18</v>
       </c>
       <c r="E43" s="19">
         <f>ROUND(C43*D43,2)</f>
@@ -1457,7 +1457,7 @@
     <row r="59" ht="36" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. La fila 'Salario base' y el % de IRPF son valores de ejemplo. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
+          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para 3.800 € brutos al mes. El 18 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Compute gross salary from target net pay in payslip template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjpH9z1P7SfaWGA8PX7UuE
</commit_message>
<xml_diff>
--- a/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
+++ b/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
@@ -119,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,13 +129,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -144,7 +151,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -153,7 +159,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -248,9 +253,14 @@
     <author>Plantilla</author>
   </authors>
   <commentList>
+    <comment ref="J4" authorId="0" shapeId="0">
+      <text>
+        <t>Base máxima de cotización 2026. Comprobar en la Orden de cotización del año.</t>
+      </text>
+    </comment>
     <comment ref="B22" authorId="0" shapeId="0">
       <text>
-        <t>Salario bruto mensual de 3.800 €. Si se reparte en varios conceptos (complementos, prorrata de pagas), ajusta estas filas para que sumen lo pactado en el contrato.</t>
+        <t>Se calcula a partir del líquido deseado (celda J3). Si se reparte en varios conceptos (complementos, prorrata de pagas), ajusta estas filas para que sumen lo pactado en el contrato.</t>
       </text>
     </comment>
     <comment ref="B28" authorId="0" shapeId="0">
@@ -581,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -591,6 +601,8 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,6 +641,21 @@
           <t>EUR</t>
         </is>
       </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Cálculo del bruto (no se imprime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Líquido deseado</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>3800</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -636,82 +663,133 @@
           <t>Datos de la empresa</t>
         </is>
       </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Base máxima cotización (mensual)</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>5101.2</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Domicilio</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>CIF</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>% Seguridad Social trabajador</t>
+        </is>
+      </c>
+      <c r="J5" s="9">
+        <f>SUM(D39:D42)</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Club Deportivo ESD Hoops</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>C/ Pedro Cabrera Hernández, nº 3, Oficina 3, Barrio Contrapeso, 35215</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>G93916039</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>% IRPF</t>
+        </is>
+      </c>
+      <c r="J6" s="9">
+        <f>D43</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Nº Inscripción SS (CCC)</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Convenio aplicable</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Mes/Año</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Bruto necesario</t>
+        </is>
+      </c>
+      <c r="J7" s="11">
+        <f>ROUND(IF(J3/(1-J5-J6)&lt;=J4,J3/(1-J5-J6),(J3+J5*J4)/(1-J6)),2)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="12" t="inlineStr"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>09/2026</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Comprobación: líquido resultante</t>
+        </is>
+      </c>
+      <c r="J8" s="13">
+        <f>E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>El salario base (D22) se calcula solo a partir del líquido deseado. Si añades otros conceptos, quita la fórmula de D22 y reparte a mano.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -721,183 +799,184 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Empleado</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Domicilio</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>DNI / NIE</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n"/>
+      <c r="G11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="9" t="inlineStr"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="A12" s="12" t="inlineStr"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="12" t="inlineStr"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="12" t="inlineStr"/>
+      <c r="G12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Nº Personal</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Categoría / Puesto</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Antigüedad</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n"/>
+      <c r="G13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="9" t="inlineStr"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="9" t="inlineStr"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="A14" s="12" t="inlineStr"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="12" t="inlineStr"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="12" t="inlineStr"/>
+      <c r="G14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Grupo Profesional</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Grupo de Cotización</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Nº Afiliación SS</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
+      <c r="G15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="9" t="inlineStr"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="9" t="inlineStr"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="A16" s="12" t="inlineStr"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="12" t="inlineStr"/>
+      <c r="G16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Tipo de contrato</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Indefinido</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="7" t="inlineStr"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="6" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Unidades</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>Precio/Ud.</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>Devengo</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>Cotiza SS</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>Tributa IRPF</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Devengos (percepciones):</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Salario base mensual</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="14" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E22" s="15">
+      <c r="D22" s="6">
+        <f>$J$7</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
         <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),C22*D22,0)</f>
         <v/>
       </c>
@@ -913,19 +992,19 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Complemento de puesto</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="15">
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="19">
         <f>IF(AND(C23&lt;&gt;"",D23&lt;&gt;""),C23*D23,0)</f>
         <v/>
       </c>
@@ -941,19 +1020,19 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>003</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Plus de transporte</t>
         </is>
       </c>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="15">
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="19">
         <f>IF(AND(C24&lt;&gt;"",D24&lt;&gt;""),C24*D24,0)</f>
         <v/>
       </c>
@@ -969,19 +1048,19 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>004</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Horas extraordinarias</t>
         </is>
       </c>
-      <c r="C25" s="13" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="15">
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="19">
         <f>IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),C25*D25,0)</f>
         <v/>
       </c>
@@ -997,19 +1076,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>005</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Prorrata pagas extraordinarias</t>
         </is>
       </c>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="15">
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="19">
         <f>IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),C26*D26,0)</f>
         <v/>
       </c>
@@ -1025,19 +1104,19 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>006</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Incentivos / primas por objetivos</t>
         </is>
       </c>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="15">
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="19">
         <f>IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),C27*D27,0)</f>
         <v/>
       </c>
@@ -1053,19 +1132,19 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>007</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Dietas y gastos de viaje (exentas)</t>
         </is>
       </c>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="15">
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="19">
         <f>IF(AND(C28&lt;&gt;"",D28&lt;&gt;""),C28*D28,0)</f>
         <v/>
       </c>
@@ -1081,15 +1160,15 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>008</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="15">
+      <c r="B29" s="12" t="inlineStr"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="19">
         <f>IF(AND(C29&lt;&gt;"",D29&lt;&gt;""),C29*D29,0)</f>
         <v/>
       </c>
@@ -1105,15 +1184,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>009</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="15">
+      <c r="B30" s="12" t="inlineStr"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="19">
         <f>IF(AND(C30&lt;&gt;"",D30&lt;&gt;""),C30*D30,0)</f>
         <v/>
       </c>
@@ -1129,15 +1208,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>010</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr"/>
-      <c r="C31" s="13" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="15">
+      <c r="B31" s="12" t="inlineStr"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="19">
         <f>IF(AND(C31&lt;&gt;"",D31&lt;&gt;""),C31*D31,0)</f>
         <v/>
       </c>
@@ -1153,222 +1232,222 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>TOTAL DEVENGADO</t>
         </is>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="21">
         <f>SUM(E22:E31)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Bases:</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>Base de cotización Seguridad Social</t>
         </is>
       </c>
-      <c r="E35" s="19">
-        <f>SUMIF(F22:F31,"S",E22:E31)</f>
+      <c r="E35" s="13">
+        <f>MIN(SUMIF(F22:F31,"S",E22:E31),$J$4)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>Base sujeta a IRPF</t>
         </is>
       </c>
-      <c r="E36" s="19">
+      <c r="E36" s="13">
         <f>SUMIF(G22:G31,"S",E22:E31)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>Deducciones</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D38" s="10" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>Tipo %</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="15" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>/350</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Contingencias comunes</t>
         </is>
       </c>
-      <c r="C39" s="19">
+      <c r="C39" s="13">
         <f>E35</f>
         <v/>
       </c>
-      <c r="D39" s="20" t="n">
+      <c r="D39" s="23" t="n">
         <v>0.047</v>
       </c>
-      <c r="E39" s="19">
+      <c r="E39" s="13">
         <f>ROUND(C39*D39,2)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>/355</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Mecanismo Equidad Intergeneracional (MEI)</t>
         </is>
       </c>
-      <c r="C40" s="19">
+      <c r="C40" s="13">
         <f>E35</f>
         <v/>
       </c>
-      <c r="D40" s="20" t="n">
+      <c r="D40" s="23" t="n">
         <v>0.0015</v>
       </c>
-      <c r="E40" s="19">
+      <c r="E40" s="13">
         <f>ROUND(C40*D40,2)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>/370</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Desempleo</t>
         </is>
       </c>
-      <c r="C41" s="19">
+      <c r="C41" s="13">
         <f>E35</f>
         <v/>
       </c>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="23" t="n">
         <v>0.0155</v>
       </c>
-      <c r="E41" s="19">
+      <c r="E41" s="13">
         <f>ROUND(C41*D41,2)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>/380</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Formación profesional</t>
         </is>
       </c>
-      <c r="C42" s="19">
+      <c r="C42" s="13">
         <f>E35</f>
         <v/>
       </c>
-      <c r="D42" s="20" t="n">
+      <c r="D42" s="23" t="n">
         <v>0.001</v>
       </c>
-      <c r="E42" s="19">
+      <c r="E42" s="13">
         <f>ROUND(C42*D42,2)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>/400</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Retención IRPF</t>
         </is>
       </c>
-      <c r="C43" s="19">
+      <c r="C43" s="13">
         <f>E36</f>
         <v/>
       </c>
-      <c r="D43" s="20" t="n">
+      <c r="D43" s="23" t="n">
         <v>0.18</v>
       </c>
-      <c r="E43" s="19">
+      <c r="E43" s="13">
         <f>ROUND(C43*D43,2)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>/500</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Anticipos / otras deducciones</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr"/>
-      <c r="D44" s="7" t="inlineStr"/>
-      <c r="E44" s="21" t="n">
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>TOTAL A DEDUCIR</t>
         </is>
       </c>
-      <c r="E45" s="17">
+      <c r="E45" s="21">
         <f>SUM(E39:E44)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="inlineStr">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>LÍQUIDO A PERCIBIR</t>
         </is>
       </c>
-      <c r="E47" s="23">
+      <c r="E47" s="26">
         <f>E32-E45</f>
         <v/>
       </c>
@@ -1381,88 +1460,88 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Entidad</t>
         </is>
       </c>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>IBAN</t>
         </is>
       </c>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Fecha de pago</t>
         </is>
       </c>
-      <c r="G50" s="6" t="n"/>
+      <c r="G50" s="8" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="9" t="inlineStr"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="9" t="inlineStr"/>
-      <c r="G51" s="6" t="n"/>
+      <c r="A51" s="12" t="inlineStr"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="12" t="inlineStr"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="12" t="inlineStr"/>
+      <c r="G51" s="8" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="24" t="inlineStr">
+      <c r="A53" s="27" t="inlineStr">
         <is>
           <t>Firma y sello de la empresa</t>
         </is>
       </c>
-      <c r="E53" s="24" t="inlineStr">
+      <c r="E53" s="27" t="inlineStr">
         <is>
           <t>Recibí del trabajador</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="6" t="n"/>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="6" t="n"/>
-      <c r="E56" s="6" t="n"/>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="6" t="n"/>
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="8" t="n"/>
     </row>
     <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para 3.800 € brutos al mes. El 18 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para un líquido de 3.800 € al mes (el bruto se calcula en J7). El 18 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="57">
+  <mergeCells count="59">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="C50:E50"/>
@@ -1472,8 +1551,10 @@
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A51:B51"/>
+    <mergeCell ref="I2:J2"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="I9:J11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A10:G10"/>

</xml_diff>

<commit_message>
Split gross salary into payslip concepts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjpH9z1P7SfaWGA8PX7UuE
</commit_message>
<xml_diff>
--- a/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
+++ b/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
@@ -18,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;;-#,##0.00 &quot;€&quot;;&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00 &quot;€&quot;;-#,##0.00 &quot;€&quot;;&quot;0,00 €&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -119,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -140,6 +141,8 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -260,7 +263,7 @@
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
       <text>
-        <t>Se calcula a partir del líquido deseado (celda J3). Si se reparte en varios conceptos (complementos, prorrata de pagas), ajusta estas filas para que sumen lo pactado en el contrato.</t>
+        <t>Se calcula a partir del bruto necesario (J7) y el reparto de J13:J14. Si se reparte en varios conceptos (complementos, prorrata de pagas), ajusta estas filas para que sumen lo pactado en el contrato.</t>
       </text>
     </comment>
     <comment ref="B28" authorId="0" shapeId="0">
@@ -784,13 +787,6 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>El salario base (D22) se calcula solo a partir del líquido deseado. Si añades otros conceptos, quita la fórmula de D22 y reparte a mano.</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -818,6 +814,11 @@
         </is>
       </c>
       <c r="G11" s="8" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Reparto del bruto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr"/>
@@ -827,6 +828,16 @@
       <c r="E12" s="8" t="n"/>
       <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="8" t="n"/>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Criterio</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Editable</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -848,6 +859,14 @@
         </is>
       </c>
       <c r="G13" s="8" t="n"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Plus de transporte (fijo)</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr"/>
@@ -857,6 +876,14 @@
       <c r="E14" s="8" t="n"/>
       <c r="F14" s="12" t="inlineStr"/>
       <c r="G14" s="8" t="n"/>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>% (bruto − transporte) para base + prorrata</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -878,6 +905,15 @@
         </is>
       </c>
       <c r="G15" s="8" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Suma de conceptos</t>
+        </is>
+      </c>
+      <c r="J15" s="13">
+        <f>E32</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr"/>
@@ -887,6 +923,15 @@
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="12" t="inlineStr"/>
       <c r="G16" s="8" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Diferencia con bruto necesario</t>
+        </is>
+      </c>
+      <c r="J16" s="15">
+        <f>J7-E32</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -900,6 +945,11 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="7" t="inlineStr"/>
       <c r="G17" s="8" t="n"/>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Salario base = (bruto − transporte) × % ÷ 7/6. Prorrata = 2 pagas extra de salario base ÷ 12. Complemento de puesto = lo que falta hasta el bruto, para que cuadre al céntimo. Ajusta el reparto al contrato o convenio.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -914,69 +964,70 @@
       <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="8" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Unidades</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Precio/Ud.</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Devengo</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Cotiza SS</t>
         </is>
       </c>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Tributa IRPF</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Devengos (percepciones):</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>Salario base mensual</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="n">
+          <t>Salario base</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="6">
-        <f>$J$7</f>
-        <v/>
-      </c>
-      <c r="E22" s="19">
+      <c r="D22" s="13">
+        <f>ROUND(($J$7-$J$13)*$J$14/(7/6),2)</f>
+        <v/>
+      </c>
+      <c r="E22" s="21">
         <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),C22*D22,0)</f>
         <v/>
       </c>
@@ -992,7 +1043,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>002</t>
         </is>
@@ -1002,9 +1053,14 @@
           <t>Complemento de puesto</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="19">
+      <c r="C23" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="13">
+        <f>$J$7-D22-D24-D26</f>
+        <v/>
+      </c>
+      <c r="E23" s="21">
         <f>IF(AND(C23&lt;&gt;"",D23&lt;&gt;""),C23*D23,0)</f>
         <v/>
       </c>
@@ -1020,7 +1076,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>003</t>
         </is>
@@ -1030,9 +1086,14 @@
           <t>Plus de transporte</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="19">
+      <c r="C24" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="13">
+        <f>$J$13</f>
+        <v/>
+      </c>
+      <c r="E24" s="21">
         <f>IF(AND(C24&lt;&gt;"",D24&lt;&gt;""),C24*D24,0)</f>
         <v/>
       </c>
@@ -1048,7 +1109,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>004</t>
         </is>
@@ -1058,9 +1119,9 @@
           <t>Horas extraordinarias</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n"/>
+      <c r="C25" s="20" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="19">
+      <c r="E25" s="21">
         <f>IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),C25*D25,0)</f>
         <v/>
       </c>
@@ -1076,7 +1137,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>005</t>
         </is>
@@ -1086,9 +1147,14 @@
           <t>Prorrata pagas extraordinarias</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="19">
+      <c r="C26" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="13">
+        <f>ROUND(D22*2/12,2)</f>
+        <v/>
+      </c>
+      <c r="E26" s="21">
         <f>IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),C26*D26,0)</f>
         <v/>
       </c>
@@ -1104,7 +1170,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>006</t>
         </is>
@@ -1114,9 +1180,9 @@
           <t>Incentivos / primas por objetivos</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n"/>
+      <c r="C27" s="20" t="n"/>
       <c r="D27" s="6" t="n"/>
-      <c r="E27" s="19">
+      <c r="E27" s="21">
         <f>IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),C27*D27,0)</f>
         <v/>
       </c>
@@ -1132,7 +1198,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>007</t>
         </is>
@@ -1142,9 +1208,9 @@
           <t>Dietas y gastos de viaje (exentas)</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n"/>
+      <c r="C28" s="20" t="n"/>
       <c r="D28" s="6" t="n"/>
-      <c r="E28" s="19">
+      <c r="E28" s="21">
         <f>IF(AND(C28&lt;&gt;"",D28&lt;&gt;""),C28*D28,0)</f>
         <v/>
       </c>
@@ -1160,15 +1226,15 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>008</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr"/>
-      <c r="C29" s="18" t="n"/>
+      <c r="C29" s="20" t="n"/>
       <c r="D29" s="6" t="n"/>
-      <c r="E29" s="19">
+      <c r="E29" s="21">
         <f>IF(AND(C29&lt;&gt;"",D29&lt;&gt;""),C29*D29,0)</f>
         <v/>
       </c>
@@ -1184,15 +1250,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>009</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr"/>
-      <c r="C30" s="18" t="n"/>
+      <c r="C30" s="20" t="n"/>
       <c r="D30" s="6" t="n"/>
-      <c r="E30" s="19">
+      <c r="E30" s="21">
         <f>IF(AND(C30&lt;&gt;"",D30&lt;&gt;""),C30*D30,0)</f>
         <v/>
       </c>
@@ -1208,15 +1274,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>010</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr"/>
-      <c r="C31" s="18" t="n"/>
+      <c r="C31" s="20" t="n"/>
       <c r="D31" s="6" t="n"/>
-      <c r="E31" s="19">
+      <c r="E31" s="21">
         <f>IF(AND(C31&lt;&gt;"",D31&lt;&gt;""),C31*D31,0)</f>
         <v/>
       </c>
@@ -1232,25 +1298,25 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>TOTAL DEVENGADO</t>
         </is>
       </c>
-      <c r="E32" s="21">
+      <c r="E32" s="23">
         <f>SUM(E22:E31)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Bases:</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>Base de cotización Seguridad Social</t>
         </is>
@@ -1261,7 +1327,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>Base sujeta a IRPF</t>
         </is>
@@ -1272,34 +1338,34 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>Deducciones</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>Tipo %</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>/350</t>
         </is>
@@ -1313,7 +1379,7 @@
         <f>E35</f>
         <v/>
       </c>
-      <c r="D39" s="23" t="n">
+      <c r="D39" s="25" t="n">
         <v>0.047</v>
       </c>
       <c r="E39" s="13">
@@ -1322,7 +1388,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>/355</t>
         </is>
@@ -1336,7 +1402,7 @@
         <f>E35</f>
         <v/>
       </c>
-      <c r="D40" s="23" t="n">
+      <c r="D40" s="25" t="n">
         <v>0.0015</v>
       </c>
       <c r="E40" s="13">
@@ -1345,7 +1411,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>/370</t>
         </is>
@@ -1359,7 +1425,7 @@
         <f>E35</f>
         <v/>
       </c>
-      <c r="D41" s="23" t="n">
+      <c r="D41" s="25" t="n">
         <v>0.0155</v>
       </c>
       <c r="E41" s="13">
@@ -1368,7 +1434,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>/380</t>
         </is>
@@ -1382,7 +1448,7 @@
         <f>E35</f>
         <v/>
       </c>
-      <c r="D42" s="23" t="n">
+      <c r="D42" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="E42" s="13">
@@ -1391,7 +1457,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>/400</t>
         </is>
@@ -1405,7 +1471,7 @@
         <f>E36</f>
         <v/>
       </c>
-      <c r="D43" s="23" t="n">
+      <c r="D43" s="25" t="n">
         <v>0.18</v>
       </c>
       <c r="E43" s="13">
@@ -1414,7 +1480,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>/500</t>
         </is>
@@ -1426,28 +1492,28 @@
       </c>
       <c r="C44" s="5" t="inlineStr"/>
       <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="24" t="n">
+      <c r="E44" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="20" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>TOTAL A DEDUCIR</t>
         </is>
       </c>
-      <c r="E45" s="21">
+      <c r="E45" s="23">
         <f>SUM(E39:E44)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25" t="inlineStr">
+      <c r="A47" s="27" t="inlineStr">
         <is>
           <t>LÍQUIDO A PERCIBIR</t>
         </is>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="28">
         <f>E32-E45</f>
         <v/>
       </c>
@@ -1490,12 +1556,12 @@
       <c r="G51" s="8" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="27" t="inlineStr">
+      <c r="A53" s="29" t="inlineStr">
         <is>
           <t>Firma y sello de la empresa</t>
         </is>
       </c>
-      <c r="E53" s="27" t="inlineStr">
+      <c r="E53" s="29" t="inlineStr">
         <is>
           <t>Recibí del trabajador</t>
         </is>
@@ -1534,14 +1600,14 @@
       <c r="G57" s="8" t="n"/>
     </row>
     <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="28" t="inlineStr">
+      <c r="A59" s="30" t="inlineStr">
         <is>
           <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para un líquido de 3.800 € al mes (el bruto se calcula en J7). El 18 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="59">
+  <mergeCells count="60">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="C50:E50"/>
@@ -1553,13 +1619,14 @@
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="I9:J11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="C51:E51"/>
+    <mergeCell ref="I17:J20"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="F12:G12"/>

</xml_diff>

<commit_message>
Add employer social security contributions and solidarity quota to payslip template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjpH9z1P7SfaWGA8PX7UuE
</commit_message>
<xml_diff>
--- a/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
+++ b/nominas/Plantilla_Nomina_ESD_Hoops.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nómina" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Nómina'!$A$1:$G$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Nómina'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -276,29 +276,69 @@
         <t>Suma de conceptos marcados 'S' en Cotiza SS. Comprobar que no queda por debajo de la base mínima del grupo de cotización.</t>
       </text>
     </comment>
-    <comment ref="D39" authorId="0" shapeId="0">
+    <comment ref="D40" authorId="0" shapeId="0">
       <text>
         <t>Tipo trabajador 4,70 %. Revisar cada año.</t>
       </text>
     </comment>
-    <comment ref="D40" authorId="0" shapeId="0">
+    <comment ref="D41" authorId="0" shapeId="0">
       <text>
         <t>MEI a cargo del trabajador: 0,15 % en 2026 (0,13 % en 2025). Revisar cada año.</t>
       </text>
     </comment>
-    <comment ref="D41" authorId="0" shapeId="0">
+    <comment ref="D42" authorId="0" shapeId="0">
       <text>
         <t>1,55 % contrato indefinido; 1,60 % contrato temporal.</t>
       </text>
     </comment>
-    <comment ref="D42" authorId="0" shapeId="0">
+    <comment ref="D43" authorId="0" shapeId="0">
       <text>
         <t>0,10 % a cargo del trabajador.</t>
       </text>
     </comment>
-    <comment ref="D43" authorId="0" shapeId="0">
+    <comment ref="D44" authorId="0" shapeId="0">
       <text>
-        <t>18 % orientativo. Calcular con el simulador de retenciones de la AEAT según la situación del trabajador.</t>
+        <t>Parte del trabajador de la cuota de solidaridad (2026: 1,15 % total en el primer tramo, ~0,19 % a cargo del trabajador). Solo se aplica a lo que supera la base máxima. Comprobar cada año.</t>
+      </text>
+    </comment>
+    <comment ref="D45" authorId="0" shapeId="0">
+      <text>
+        <t>25 % orientativo. Calcular con el simulador de retenciones de la AEAT según la situación del trabajador.</t>
+      </text>
+    </comment>
+    <comment ref="D53" authorId="0" shapeId="0">
+      <text>
+        <t>23,60 % a cargo de la empresa.</t>
+      </text>
+    </comment>
+    <comment ref="D54" authorId="0" shapeId="0">
+      <text>
+        <t>MEI empresa: 0,75 % en 2026 (0,67 % en 2025).</t>
+      </text>
+    </comment>
+    <comment ref="D55" authorId="0" shapeId="0">
+      <text>
+        <t>5,50 % contrato indefinido; 6,70 % contrato temporal.</t>
+      </text>
+    </comment>
+    <comment ref="D56" authorId="0" shapeId="0">
+      <text>
+        <t>0,20 %.</t>
+      </text>
+    </comment>
+    <comment ref="D57" authorId="0" shapeId="0">
+      <text>
+        <t>0,60 %.</t>
+      </text>
+    </comment>
+    <comment ref="D58" authorId="0" shapeId="0">
+      <text>
+        <t>Depende de la actividad (CNAE) y del puesto. 3,30 % orientativo para actividades deportivas (CNAE 93); 1,50 % si el trabajo es exclusivamente de oficina. Comprobar con la tarifa de primas vigente.</t>
+      </text>
+    </comment>
+    <comment ref="D59" authorId="0" shapeId="0">
+      <text>
+        <t>Parte de la empresa de la cuota de solidaridad (~0,96 % en 2026, primer tramo). Comprobar cada año.</t>
       </text>
     </comment>
   </commentList>
@@ -594,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -701,7 +741,7 @@
         </is>
       </c>
       <c r="J5" s="9">
-        <f>SUM(D39:D42)</f>
+        <f>SUM(D40:D43)</f>
         <v/>
       </c>
     </row>
@@ -731,7 +771,7 @@
         </is>
       </c>
       <c r="J6" s="9">
-        <f>D43</f>
+        <f>D45</f>
         <v/>
       </c>
     </row>
@@ -761,7 +801,7 @@
         </is>
       </c>
       <c r="J7" s="11">
-        <f>ROUND(IF(J3/(1-J5-J6)&lt;=J4,J3/(1-J5-J6),(J3+J5*J4)/(1-J6)),2)</f>
+        <f>ROUND(IF(J3/(1-J5-J6)&lt;=J4,J3/(1-J5-J6),(J3+J5*J4-J8*J4)/(1-J6-J8)),2)</f>
         <v/>
       </c>
     </row>
@@ -779,11 +819,22 @@
       <c r="G8" s="8" t="n"/>
       <c r="I8" s="5" t="inlineStr">
         <is>
+          <t>% solidaridad trabajador</t>
+        </is>
+      </c>
+      <c r="J8" s="9">
+        <f>D44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="I9" s="5" t="inlineStr">
+        <is>
           <t>Comprobación: líquido resultante</t>
         </is>
       </c>
-      <c r="J8" s="13">
-        <f>E47</f>
+      <c r="J9" s="13">
+        <f>E49</f>
         <v/>
       </c>
     </row>
@@ -1337,65 +1388,53 @@
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>Exceso sobre base máxima (cuota de solidaridad)</t>
+        </is>
+      </c>
+      <c r="E37" s="21">
+        <f>MAX(0,SUMIF(F22:F31,"S",E22:E31)-$J$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Deducciones</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>Tipo %</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>/350</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Contingencias comunes</t>
-        </is>
-      </c>
-      <c r="C39" s="13">
-        <f>E35</f>
-        <v/>
-      </c>
-      <c r="D39" s="25" t="n">
-        <v>0.047</v>
-      </c>
-      <c r="E39" s="13">
-        <f>ROUND(C39*D39,2)</f>
-        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>/355</t>
+          <t>/350</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Mecanismo Equidad Intergeneracional (MEI)</t>
+          <t>Contingencias comunes</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -1403,7 +1442,7 @@
         <v/>
       </c>
       <c r="D40" s="25" t="n">
-        <v>0.0015</v>
+        <v>0.047</v>
       </c>
       <c r="E40" s="13">
         <f>ROUND(C40*D40,2)</f>
@@ -1413,12 +1452,12 @@
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>/370</t>
+          <t>/355</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Desempleo</t>
+          <t>Mecanismo Equidad Intergeneracional (MEI)</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -1426,7 +1465,7 @@
         <v/>
       </c>
       <c r="D41" s="25" t="n">
-        <v>0.0155</v>
+        <v>0.0015</v>
       </c>
       <c r="E41" s="13">
         <f>ROUND(C41*D41,2)</f>
@@ -1436,12 +1475,12 @@
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>/380</t>
+          <t>/370</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Formación profesional</t>
+          <t>Desempleo</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -1449,7 +1488,7 @@
         <v/>
       </c>
       <c r="D42" s="25" t="n">
-        <v>0.001</v>
+        <v>0.0155</v>
       </c>
       <c r="E42" s="13">
         <f>ROUND(C42*D42,2)</f>
@@ -1459,20 +1498,20 @@
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>/400</t>
+          <t>/380</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Retención IRPF</t>
+          <t>Formación profesional</t>
         </is>
       </c>
       <c r="C43" s="13">
-        <f>E36</f>
+        <f>E35</f>
         <v/>
       </c>
       <c r="D43" s="25" t="n">
-        <v>0.18</v>
+        <v>0.001</v>
       </c>
       <c r="E43" s="13">
         <f>ROUND(C43*D43,2)</f>
@@ -1482,141 +1521,403 @@
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
+          <t>/360</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Cuota de solidaridad</t>
+        </is>
+      </c>
+      <c r="C44" s="13">
+        <f>E37</f>
+        <v/>
+      </c>
+      <c r="D44" s="25" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="E44" s="13">
+        <f>ROUND(C44*D44,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>/400</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Retención IRPF</t>
+        </is>
+      </c>
+      <c r="C45" s="13">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="D45" s="25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E45" s="13">
+        <f>ROUND(C45*D45,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
           <t>/500</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Anticipos / otras deducciones</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr"/>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="26" t="n">
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="26" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>TOTAL A DEDUCIR</t>
         </is>
       </c>
-      <c r="E45" s="23">
-        <f>SUM(E39:E44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="27" t="inlineStr">
+      <c r="E47" s="23">
+        <f>SUM(E40:E46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
         <is>
           <t>LÍQUIDO A PERCIBIR</t>
         </is>
       </c>
-      <c r="E47" s="28">
-        <f>E32-E45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="E49" s="28">
+        <f>E32-E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Aportación de la empresa a la Seguridad Social (informativo, no se descuenta al trabajador)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Tipo %</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Importe</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>E350</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Contingencias comunes</t>
+        </is>
+      </c>
+      <c r="C53" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D53" s="25" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="E53" s="21">
+        <f>ROUND(C53*D53,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>E355</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Mecanismo Equidad Intergeneracional (MEI)</t>
+        </is>
+      </c>
+      <c r="C54" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D54" s="25" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="E54" s="21">
+        <f>ROUND(C54*D54,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>E370</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Desempleo</t>
+        </is>
+      </c>
+      <c r="C55" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="E55" s="21">
+        <f>ROUND(C55*D55,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>E375</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>FOGASA</t>
+        </is>
+      </c>
+      <c r="C56" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D56" s="25" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E56" s="21">
+        <f>ROUND(C56*D56,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>E380</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Formación profesional</t>
+        </is>
+      </c>
+      <c r="C57" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D57" s="25" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="E57" s="21">
+        <f>ROUND(C57*D57,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="26" customHeight="1">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>E390</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Accidentes de trabajo y enfermedad profesional (AT/EP)</t>
+        </is>
+      </c>
+      <c r="C58" s="13">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D58" s="25" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="E58" s="21">
+        <f>ROUND(C58*D58,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>E360</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Cuota de solidaridad (empresa)</t>
+        </is>
+      </c>
+      <c r="C59" s="13">
+        <f>E37</f>
+        <v/>
+      </c>
+      <c r="D59" s="25" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="E59" s="21">
+        <f>ROUND(C59*D59,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL APORTACIÓN EMPRESA</t>
+        </is>
+      </c>
+      <c r="E60" s="23">
+        <f>SUM(E53:E59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="22" t="inlineStr">
+        <is>
+          <t>COSTE TOTAL PARA LA EMPRESA (bruto + aportación)</t>
+        </is>
+      </c>
+      <c r="E61" s="23">
+        <f>E32+E60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>Entidad</t>
         </is>
       </c>
-      <c r="B50" s="8" t="n"/>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>IBAN</t>
         </is>
       </c>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="D64" s="8" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Fecha de pago</t>
         </is>
       </c>
-      <c r="G50" s="8" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr"/>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="12" t="inlineStr"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="8" t="n"/>
-      <c r="F51" s="12" t="inlineStr"/>
-      <c r="G51" s="8" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="29" t="inlineStr">
+      <c r="G64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr"/>
+      <c r="B65" s="8" t="n"/>
+      <c r="C65" s="12" t="inlineStr"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="12" t="inlineStr"/>
+      <c r="G65" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="29" t="inlineStr">
         <is>
           <t>Firma y sello de la empresa</t>
         </is>
       </c>
-      <c r="E53" s="29" t="inlineStr">
+      <c r="E67" s="29" t="inlineStr">
         <is>
           <t>Recibí del trabajador</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="8" t="n"/>
-      <c r="B54" s="8" t="n"/>
-      <c r="C54" s="8" t="n"/>
-      <c r="E54" s="8" t="n"/>
-      <c r="F54" s="8" t="n"/>
-      <c r="G54" s="8" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-      <c r="B55" s="8" t="n"/>
-      <c r="C55" s="8" t="n"/>
-      <c r="E55" s="8" t="n"/>
-      <c r="F55" s="8" t="n"/>
-      <c r="G55" s="8" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n"/>
-      <c r="B56" s="8" t="n"/>
-      <c r="C56" s="8" t="n"/>
-      <c r="E56" s="8" t="n"/>
-      <c r="F56" s="8" t="n"/>
-      <c r="G56" s="8" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="n"/>
-      <c r="B57" s="8" t="n"/>
-      <c r="C57" s="8" t="n"/>
-      <c r="E57" s="8" t="n"/>
-      <c r="F57" s="8" t="n"/>
-      <c r="G57" s="8" t="n"/>
-    </row>
-    <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="30" t="inlineStr">
-        <is>
-          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para un líquido de 3.800 € al mes (el bruto se calcula en J7). El 18 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="8" t="n"/>
+      <c r="E69" s="8" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+      <c r="E70" s="8" t="n"/>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="8" t="n"/>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="8" t="n"/>
+      <c r="G71" s="8" t="n"/>
+    </row>
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="30" t="inlineStr">
+        <is>
+          <t>Leyenda: las celdas en amarillo con texto azul se rellenan a mano; las demás se calculan solas. Preparada para un líquido de 3.800 € al mes (el bruto se calcula en J7). El 25 % de IRPF es orientativo: ajústalo al tipo que dé el simulador de la AEAT para el trabajador. Los tipos de cotización son los vigentes para el trabajador en 2026; revísalos cada año.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="64">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C50:E50"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="E54:G57"/>
+    <mergeCell ref="A64:B64"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="F65:G65"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="I11:J11"/>
@@ -1625,49 +1926,54 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="I17:J20"/>
+    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A68:C71"/>
+    <mergeCell ref="E68:G71"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="F15:G15"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="I17:J20"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F51:G51"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="F18:G18"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="A49:D49"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A51:G51"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A60:D60"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A50:B50"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A54:C57"/>
+    <mergeCell ref="A61:D61"/>
     <mergeCell ref="C13:E13"/>
-    <mergeCell ref="E53:G53"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A67:C67"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="A17:B17"/>
+    <mergeCell ref="F64:G64"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="C5:E5"/>
+    <mergeCell ref="E67:G67"/>
     <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C64:E64"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="A32:D32"/>
+    <mergeCell ref="C65:E65"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>